<commit_message>
use .env instead of key vault
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -629,7 +629,7 @@
       </c>
       <c r="R2" s="14" t="inlineStr">
         <is>
-          <t>Listed as bundle at $900</t>
+          <t>Listed as bundle at $800 (was noted as $900) on FB Marketplace (3/13). Bundle has 235 clicks as of 3/15. Carter inquired about buying floor speakers separately — awaiting David's decision.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="R3" s="17" t="inlineStr">
         <is>
-          <t>Listed as bundle at $900</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 235 clicks as of 3/15.</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="R4" s="14" t="inlineStr">
         <is>
-          <t>Listed as bundle at $900</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 235 clicks as of 3/15.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
-          <t>Listed as bundle at $900</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 235 clicks as of 3/15.</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="R7" s="17" t="inlineStr">
         <is>
-          <t>Serial number AJ123154. Serial number photo added to eBay listing 3/15.</t>
+          <t>Serial number AJ123154. Serial number photo added to eBay listing 3/15. 35 views, 5 watchers (3/15). memcg_75 asked for serial number — replied 9:18 AM. Send offer eligible on eBay.</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="R8" s="14" t="inlineStr">
         <is>
-          <t>Signed &amp; numbered (~#450). COA from Renaissance Fine Arts (Cornell Gabos, 1993). Bezalel Academy Jerusalem. Professionally double-matted and framed.</t>
+          <t>Signed &amp; numbered (~#450). COA from Renaissance Fine Arts (Cornell Gabos, 1993). Bezalel Academy Jerusalem. Professionally double-matted and framed. 1 view, 0 watchers (3/15).</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
         <v>150</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="J9" s="18" t="n"/>
       <c r="K9" s="17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="R9" s="17" t="inlineStr">
         <is>
-          <t>Dark wood frame, glass front, mirrored back, asymmetric shelves. ~24x16 inches. Brass wall-mount hardware. Best sold locally (fragile).</t>
+          <t>Dark wood frame, glass front, mirrored back, asymmetric shelves. ~24x16 inches. Brass wall-mount hardware. Best sold locally (fragile). 37 clicks on FB Marketplace as of 3/15.</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>Southwestern medallion pattern, earthy tones, includes accent pillow, dark wood legs</t>
+          <t>Southwestern medallion pattern, earthy tones, includes accent pillow, dark wood legs. 5 clicks on FB Marketplace (listed 3/15).</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="R13" s="11" t="inlineStr">
         <is>
-          <t>Curved dark wood arms, geometric taupe/rust fabric, manual pushback mechanism, high back</t>
+          <t>Curved dark wood arms, geometric taupe/rust fabric, manual pushback mechanism, high back. 5 clicks on FB Marketplace (listed 3/15).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
inventory update 2026-03-16 — Singer Featherweight sold 42 to mari88530
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -78,7 +78,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,12 @@
         <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1ECF1"/>
+        <bgColor rgb="00D1ECF1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -135,7 +141,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -208,6 +214,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -629,7 +638,7 @@
       </c>
       <c r="R2" s="14" t="inlineStr">
         <is>
-          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 237 clicks as of 3/15. Carter asked about buying floor speakers separately (1h ago) — awaiting David decision on whether to split bundle. Last checked: 2026-03-15.</t>
+          <t>Bundle listing at $800 (272 clicks on FB — strong interest). Carter asked about buying floor speakers separately — replied 3/16: '$375/pair, interested?'. David confirmed ok to sell individually. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -695,7 +704,7 @@
       </c>
       <c r="R3" s="17" t="inlineStr">
         <is>
-          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 237 clicks as of 3/15. Last checked: 2026-03-15.</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). 272 clicks on bundle. David confirmed ok to sell pieces individually if needed. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -761,7 +770,7 @@
       </c>
       <c r="R4" s="14" t="inlineStr">
         <is>
-          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 237 clicks as of 3/15. Last checked: 2026-03-15.</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). 272 clicks on bundle. David confirmed ok to sell pieces individually if needed. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -827,7 +836,7 @@
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
-          <t>Listed as bundle at $800 on FB Marketplace (3/13). Bundle has 237 clicks as of 3/15. Last checked: 2026-03-15.</t>
+          <t>Listed as bundle at $800 on FB Marketplace (3/13). 272 clicks on bundle. David confirmed ok to sell pieces individually if needed. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -935,15 +944,17 @@
       <c r="I7" s="18" t="n">
         <v>380</v>
       </c>
-      <c r="J7" s="18" t="n"/>
+      <c r="J7" s="18" t="n">
+        <v>342</v>
+      </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
           <t>eBay</t>
         </is>
       </c>
-      <c r="L7" s="19" t="inlineStr">
-        <is>
-          <t>listed</t>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>sold</t>
         </is>
       </c>
       <c r="M7" s="17" t="inlineStr">
@@ -965,7 +976,7 @@
       </c>
       <c r="R7" s="17" t="inlineStr">
         <is>
-          <t>38 views, 5 watchers (3/15). 1 offer of $200 auto-declined (below $300 floor). memcg_75 serial number question answered 9:18 AM. No new messages. Last checked: 2026-03-15.</t>
+          <t>SOLD to mari88530 (Maria Lara Rivas) for $342. Order #12-14372-41895. Ship by Thu Mar 19. Payment received Mar 16. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1048,7 @@
       </c>
       <c r="R8" s="14" t="inlineStr">
         <is>
-          <t>1 view, 0 watchers (3/15). Low engagement — listed 3/14, no offers or messages. Consider price review if no activity by 3/21. Last checked: 2026-03-15.</t>
+          <t>1 view, 0 watchers — still very low engagement 2 days in. No offers or messages. Consider price review if no activity by 3/21. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1116,7 @@
       </c>
       <c r="R9" s="17" t="inlineStr">
         <is>
-          <t>39 clicks on FB Marketplace (3/15, up from 37). No messages. Last checked: 2026-03-15.</t>
+          <t>54 clicks on listing. Merrisa Allmond asked 'is this still available?' — replied 3/16: 'Yes, still available!' Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1195,7 @@
       </c>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>6 clicks on FB Marketplace (3/15, up from 5). No messages. Last checked: 2026-03-15.</t>
+          <t>26 clicks on listing. Active — no messages today. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1254,7 @@
       </c>
       <c r="R13" s="11" t="inlineStr">
         <is>
-          <t>7 clicks on FB Marketplace (3/15, up from 5). No messages. Last checked: 2026-03-15.</t>
+          <t>15 clicks on listing. Active — no messages today. Last checked: 2026-03-16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
inventory update 2026-03-19 — FB Marketplace listings for all 7 rugs + 2 mats
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -231,6 +231,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1543,7 +1544,11 @@
       <c r="N15" s="27" t="n"/>
       <c r="O15" s="27" t="n"/>
       <c r="P15" s="27" t="n"/>
-      <c r="Q15" s="27" t="n"/>
+      <c r="Q15" s="27" t="inlineStr">
+        <is>
+          <t>items/art-glass-vase-27-12-tall-top-opening-6-wide-11-wide</t>
+        </is>
+      </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
           <t>Curiouser &amp; Curiouser dealer sticker $750 retail. Jingdezhen sang de boeuf, 4-char seal mark on base.</t>
@@ -1569,14 +1574,24 @@
           <t>eBay</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L16" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298141825438</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>items/oriental-37-12-x-56-12</t>
         </is>
       </c>
     </row>
@@ -1609,6 +1624,11 @@
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>items/stone-top-coffee-table-with-built-in-lower-shelf-matching-si</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1629,14 +1649,24 @@
           <t>eBay</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L18" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298141824552</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>items/rug-30-12-x-57</t>
         </is>
       </c>
     </row>
@@ -1656,17 +1686,27 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L19" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/4295315460740523</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-39-x-39</t>
         </is>
       </c>
     </row>
@@ -1686,17 +1726,27 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L20" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/917663117719976</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-30-x-55-12</t>
         </is>
       </c>
     </row>
@@ -1716,17 +1766,27 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L21" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1236650981995574</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-28-x-44</t>
         </is>
       </c>
     </row>
@@ -1746,17 +1806,27 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L22" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/911121191540382</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-29-x-37</t>
         </is>
       </c>
     </row>
@@ -1776,17 +1846,27 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L23" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1456069612967803</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-29-x-35</t>
         </is>
       </c>
     </row>
@@ -1809,14 +1889,24 @@
           <t>eBay</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L24" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298141797227</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>items/oriental-bag-27-x-29</t>
         </is>
       </c>
     </row>
@@ -1839,14 +1929,24 @@
           <t>eBay</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L25" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/298141796002</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-saddle-bag-each-side-is-25-x-20-12-there-are-po</t>
         </is>
       </c>
     </row>
@@ -1866,17 +1966,27 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L26" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/784453008054227</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-17-x-24</t>
         </is>
       </c>
     </row>
@@ -1896,17 +2006,27 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>eBay</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L27" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1159619476157372</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>items/oriental-rug-measure-18-x-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
listed a bunch on facebook marketplace
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -1472,12 +1472,12 @@
       <c r="J14" s="22" t="n"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>FB Marketplace / Chairish</t>
-        </is>
-      </c>
-      <c r="L14" s="25" t="inlineStr">
-        <is>
-          <t>ready</t>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L14" s="30" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -1487,7 +1487,11 @@
       </c>
       <c r="N14" s="27" t="n"/>
       <c r="O14" s="27" t="n"/>
-      <c r="P14" s="27" t="n"/>
+      <c r="P14" s="27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/875609515482127</t>
+        </is>
+      </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
           <t>items/mashad-persian-rug-11x16</t>
@@ -1531,9 +1535,9 @@
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L15" s="26" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L15" s="30" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
@@ -1543,7 +1547,11 @@
       </c>
       <c r="N15" s="27" t="n"/>
       <c r="O15" s="27" t="n"/>
-      <c r="P15" s="27" t="n"/>
+      <c r="P15" s="27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/2430087930754566</t>
+        </is>
+      </c>
       <c r="Q15" s="27" t="inlineStr">
         <is>
           <t>items/art-glass-vase-27-12-tall-top-opening-6-wide-11-wide</t>
@@ -1571,7 +1579,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>FB Marketplace</t>
         </is>
       </c>
       <c r="L16" s="32" t="inlineStr">
@@ -1586,7 +1594,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/298141825438</t>
+          <t>https://www.facebook.com/marketplace/item/1258134445860417</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1614,14 +1622,19 @@
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="L17" s="32" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1291397416387369</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1646,7 +1659,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>FB Marketplace</t>
         </is>
       </c>
       <c r="L18" s="32" t="inlineStr">
@@ -1661,7 +1674,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/298141824552</t>
+          <t>https://www.facebook.com/marketplace/item/1306171418224751</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1886,7 +1899,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>FB Marketplace</t>
         </is>
       </c>
       <c r="L24" s="32" t="inlineStr">
@@ -1901,7 +1914,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/298141797227</t>
+          <t>https://www.facebook.com/marketplace/item/864521629953555</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -1926,7 +1939,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>FB Marketplace</t>
         </is>
       </c>
       <c r="L25" s="32" t="inlineStr">
@@ -1941,7 +1954,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/298141796002</t>
+          <t>https://www.facebook.com/marketplace/item/796264936376988</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">

</xml_diff>

<commit_message>
listed and excel ready
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -747,16 +747,18 @@
       <c r="H2" s="14" t="n">
         <v>475</v>
       </c>
-      <c r="I2" s="14" t="n"/>
+      <c r="I2" s="14" t="n">
+        <v>750</v>
+      </c>
       <c r="J2" s="14" t="n"/>
       <c r="K2" s="13" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L2" s="15" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L2" s="31" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M2" s="13" t="inlineStr">
@@ -764,9 +766,17 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N2" s="13" t="n"/>
+      <c r="N2" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O2" s="13" t="n"/>
-      <c r="P2" s="13" t="n"/>
+      <c r="P2" s="13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1585020142554515</t>
+        </is>
+      </c>
       <c r="Q2" s="13" t="inlineStr">
         <is>
           <t>Items to resell/Music Equipment</t>
@@ -774,7 +784,7 @@
       </c>
       <c r="R2" s="13" t="inlineStr">
         <is>
-          <t>Old FB account - user handling separately</t>
+          <t>Listed as full system bundle with CC-370, PS-1000, and Marantz receiver. Bundle price $750.</t>
         </is>
       </c>
     </row>
@@ -813,16 +823,18 @@
       <c r="H3" s="17" t="n">
         <v>225</v>
       </c>
-      <c r="I3" s="17" t="n"/>
+      <c r="I3" s="17" t="n">
+        <v>750</v>
+      </c>
       <c r="J3" s="17" t="n"/>
       <c r="K3" s="16" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L3" s="15" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L3" s="31" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M3" s="16" t="inlineStr">
@@ -830,9 +842,17 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N3" s="16" t="n"/>
+      <c r="N3" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O3" s="16" t="n"/>
-      <c r="P3" s="16" t="n"/>
+      <c r="P3" s="16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1585020142554515</t>
+        </is>
+      </c>
       <c r="Q3" s="16" t="inlineStr">
         <is>
           <t>Items to resell/Music Equipment</t>
@@ -840,7 +860,7 @@
       </c>
       <c r="R3" s="16" t="inlineStr">
         <is>
-          <t>Old FB account - user handling separately</t>
+          <t>Bundled with Monitor 9, PS-1000, Marantz — one listing at $750.</t>
         </is>
       </c>
     </row>
@@ -879,16 +899,18 @@
       <c r="H4" s="14" t="n">
         <v>275</v>
       </c>
-      <c r="I4" s="14" t="n"/>
+      <c r="I4" s="14" t="n">
+        <v>750</v>
+      </c>
       <c r="J4" s="14" t="n"/>
       <c r="K4" s="13" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L4" s="15" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L4" s="31" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M4" s="13" t="inlineStr">
@@ -896,9 +918,17 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N4" s="13" t="n"/>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O4" s="13" t="n"/>
-      <c r="P4" s="13" t="n"/>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1585020142554515</t>
+        </is>
+      </c>
       <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Items to resell/Music Equipment</t>
@@ -906,7 +936,7 @@
       </c>
       <c r="R4" s="13" t="inlineStr">
         <is>
-          <t>Old FB account - user handling separately</t>
+          <t>Bundled with Monitor 9, CC-370, Marantz — one listing at $750.</t>
         </is>
       </c>
     </row>
@@ -945,16 +975,18 @@
       <c r="H5" s="17" t="n">
         <v>200</v>
       </c>
-      <c r="I5" s="17" t="n"/>
+      <c r="I5" s="17" t="n">
+        <v>750</v>
+      </c>
       <c r="J5" s="17" t="n"/>
       <c r="K5" s="16" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L5" s="15" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L5" s="31" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M5" s="16" t="inlineStr">
@@ -962,9 +994,17 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N5" s="16" t="n"/>
+      <c r="N5" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O5" s="16" t="n"/>
-      <c r="P5" s="16" t="n"/>
+      <c r="P5" s="16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1585020142554515</t>
+        </is>
+      </c>
       <c r="Q5" s="16" t="inlineStr">
         <is>
           <t>Items to resell/Music Equipment</t>
@@ -972,7 +1012,7 @@
       </c>
       <c r="R5" s="16" t="inlineStr">
         <is>
-          <t>Old FB account - managed from MacBook Air (bundled with Paradigm home theater)</t>
+          <t>Bundled with Paradigm Monitor 9, CC-370, PS-1000 — one listing at $750.</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1197,7 @@
       <c r="J8" s="14" t="n"/>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>eBay + FB Marketplace</t>
         </is>
       </c>
       <c r="L8" s="31" t="inlineStr">
@@ -1170,11 +1210,15 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N8" s="13" t="n"/>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="inlineStr">
         <is>
-          <t>https://www.ebay.com/itm/298122793101</t>
+          <t>https://www.facebook.com/marketplace/item/1571562920579007</t>
         </is>
       </c>
       <c r="Q8" s="13" t="inlineStr">
@@ -1182,7 +1226,11 @@
           <t>Items to resell/Painting</t>
         </is>
       </c>
-      <c r="R8" s="13" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr">
+        <is>
+          <t>Listed on both eBay and FB Marketplace. FB: https://www.facebook.com/marketplace/item/1571562920579007</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -1228,9 +1276,9 @@
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L9" s="31" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M9" s="16" t="inlineStr">
@@ -1238,9 +1286,17 @@
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="N9" s="16" t="n"/>
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O9" s="16" t="n"/>
-      <c r="P9" s="16" t="n"/>
+      <c r="P9" s="16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1616552336289478</t>
+        </is>
+      </c>
       <c r="Q9" s="16" t="inlineStr">
         <is>
           <t>Items to resell/Other Art</t>
@@ -1341,9 +1397,9 @@
           <t>FB Marketplace</t>
         </is>
       </c>
-      <c r="L12" s="24" t="inlineStr">
-        <is>
-          <t>manual</t>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>listed</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -1351,11 +1407,15 @@
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="N12" s="27" t="n"/>
+      <c r="N12" s="27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O12" s="27" t="n"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1906061356703947</t>
+          <t>https://www.facebook.com/marketplace/item/2781152878894043</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
@@ -1407,7 +1467,7 @@
       </c>
       <c r="L13" s="30" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>listed</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -1415,11 +1475,15 @@
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="N13" s="27" t="n"/>
+      <c r="N13" s="27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O13" s="27" t="n"/>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1255615856540782</t>
+          <t>https://www.facebook.com/marketplace/item/3975772839389217</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr">
@@ -1468,7 +1532,9 @@
       <c r="H14" s="23" t="n">
         <v>18000</v>
       </c>
-      <c r="I14" s="21" t="n"/>
+      <c r="I14" s="21" t="n">
+        <v>10000</v>
+      </c>
       <c r="J14" s="22" t="n"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1485,7 +1551,11 @@
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="N14" s="27" t="n"/>
+      <c r="N14" s="27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O14" s="27" t="n"/>
       <c r="P14" s="27" t="inlineStr">
         <is>
@@ -1516,7 +1586,11 @@
       </c>
       <c r="C15" s="27" t="n"/>
       <c r="D15" s="27" t="n"/>
-      <c r="E15" s="27" t="n"/>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="F15" s="23" t="n">
         <v>250</v>
       </c>
@@ -1545,7 +1619,11 @@
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="N15" s="27" t="n"/>
+      <c r="N15" s="27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
       <c r="O15" s="27" t="n"/>
       <c r="P15" s="27" t="inlineStr">
         <is>
@@ -1574,9 +1652,17 @@
           <t>Rugs &gt; Oriental &gt; Prayer Rugs</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G16" t="n">
         <v>225</v>
       </c>
+      <c r="I16" t="n">
+        <v>225</v>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1590,6 +1676,11 @@
       <c r="M16" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1614,9 +1705,17 @@
           <t>Furniture &gt; Tables &gt; Coffee Tables</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G17" t="n">
         <v>210</v>
       </c>
+      <c r="I17" t="n">
+        <v>210</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1630,6 +1729,11 @@
       <c r="M17" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1654,9 +1758,17 @@
           <t>Rugs &gt; Flatweave &gt; Handwoven</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G18" t="n">
         <v>75</v>
       </c>
+      <c r="I18" t="n">
+        <v>75</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1670,6 +1782,11 @@
       <c r="M18" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1694,9 +1811,17 @@
           <t>Rugs &gt; Kilims &gt; Geometric</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G19" t="n">
         <v>250</v>
       </c>
+      <c r="I19" t="n">
+        <v>250</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1710,6 +1835,11 @@
       <c r="M19" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -1734,9 +1864,17 @@
           <t>Rugs &gt; Oriental &gt; Turkish</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G20" t="n">
         <v>195</v>
       </c>
+      <c r="I20" t="n">
+        <v>195</v>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1750,6 +1888,11 @@
       <c r="M20" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -1774,9 +1917,17 @@
           <t>Rugs &gt; Kilims &gt; Geometric</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G21" t="n">
         <v>140</v>
       </c>
+      <c r="I21" t="n">
+        <v>140</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1790,6 +1941,11 @@
       <c r="M21" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -1814,9 +1970,17 @@
           <t>Rugs &gt; Oriental &gt; Persian</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G22" t="n">
         <v>250</v>
       </c>
+      <c r="I22" t="n">
+        <v>250</v>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1830,6 +1994,11 @@
       <c r="M22" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -1854,9 +2023,17 @@
           <t>Rugs &gt; Oriental &gt; Persian</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G23" t="n">
         <v>285</v>
       </c>
+      <c r="I23" t="n">
+        <v>285</v>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1870,6 +2047,11 @@
       <c r="M23" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -1894,9 +2076,17 @@
           <t>Rugs &gt; Tribal Bags &gt; Baluchi</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G24" t="n">
         <v>225</v>
       </c>
+      <c r="I24" t="n">
+        <v>225</v>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1910,6 +2100,11 @@
       <c r="M24" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -1934,9 +2129,17 @@
           <t>Rugs &gt; Tribal Bags &gt; Khorjin</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G25" t="n">
         <v>375</v>
       </c>
+      <c r="I25" t="n">
+        <v>375</v>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1950,6 +2153,11 @@
       <c r="M25" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -1974,9 +2182,17 @@
           <t>Rugs &gt; Oriental &gt; Baluchi</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G26" t="n">
         <v>75</v>
       </c>
+      <c r="I26" t="n">
+        <v>75</v>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -1990,6 +2206,11 @@
       <c r="M26" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2014,9 +2235,17 @@
           <t>Rugs &gt; Oriental &gt; Floral</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Used - Good</t>
+        </is>
+      </c>
       <c r="G27" t="n">
         <v>65</v>
       </c>
+      <c r="I27" t="n">
+        <v>65</v>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>FB Marketplace</t>
@@ -2030,6 +2259,11 @@
       <c r="M27" t="inlineStr">
         <is>
           <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">

</xml_diff>

<commit_message>
update summary excel page
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0_);($#,##0)"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,13 @@
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -136,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -232,6 +239,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2288,99 +2297,182 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28.005" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
-    <col width="15.005" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
+    <col width="30" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
+    <col width="20" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>Resell Inventory Summary</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="7" t="n"/>
-      <c r="B2" s="8" t="n"/>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Last Updated:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1"/>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>COUNTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Total Items:</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <f>COUNTA(Inventory!A2:A9)</f>
+      <c r="B5">
+        <f>COUNTA(Inventory!A2:A25)-COUNTIF(Inventory!A2:A25,"TOTALS")</f>
         <v/>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Listed:</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <f>COUNTIF(Inventory!L2:L9,"listed")</f>
+      <c r="B6">
+        <f>COUNTIF(Inventory!L2:L25,"listed")</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Sold:</t>
         </is>
       </c>
-      <c r="B5" s="5">
-        <f>COUNTIF(Inventory!L2:L9,"sold")</f>
+      <c r="B7">
+        <f>COUNTIF(Inventory!L2:L25,"sold")</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Draft:</t>
         </is>
       </c>
-      <c r="B6" s="5">
-        <f>COUNTIF(Inventory!L2:L9,"draft")</f>
+      <c r="B8">
+        <f>COUNTIF(Inventory!L2:L25,"draft")</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Est. Total (Quick Sale):</t>
-        </is>
-      </c>
-      <c r="B7" s="6">
-        <f>SUM(Inventory!F2:F9)</f>
+    <row r="9" ht="15" customHeight="1"/>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>VALUATIONS (active listings only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Quick Sale Total:</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>SUMIF(Inventory!L2:L25,"listed",Inventory!F2:F25)</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Est. Total (Market):</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>SUM(Inventory!G2:G9)</f>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Market Price Total:</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>SUMIF(Inventory!L2:L25,"listed",Inventory!G2:G25)</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Est. Total (Optimistic):</t>
-        </is>
-      </c>
-      <c r="B9" s="6">
-        <f>SUM(Inventory!H2:H9)</f>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Optimistic Total:</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>SUMIF(Inventory!L2:L25,"listed",Inventory!H2:H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>SOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Total Sold Revenue:</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>SUMIF(Inventory!L2:L25,"sold",Inventory!J2:J25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>PLATFORMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>On FB Marketplace:</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>COUNTIFS(Inventory!K2:K25,"FB Marketplace",Inventory!L2:L25,"listed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>On eBay:</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>COUNTIFS(Inventory!K2:K25,"eBay",Inventory!L2:L25,"listed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>On Both:</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>COUNTIFS(Inventory!K2:K25,"eBay + FB Marketplace",Inventory!L2:L25,"listed")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
inventory update 2026-03-20 — add chinese-floral-mat-18x24 draft
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resell_inventory.xlsx
+++ b/resell_inventory.xlsx
@@ -65,7 +65,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +108,12 @@
         <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+        <bgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -143,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -241,6 +247,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,7 +613,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.005" bestFit="1" customWidth="1" style="7" min="1" max="1"/>
@@ -2286,6 +2293,55 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chinese Floral Wool Scatter Mat 18x24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rugs / Home Decor</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>50</v>
+      </c>
+      <c r="G28" t="n">
+        <v>95</v>
+      </c>
+      <c r="H28" t="n">
+        <v>150</v>
+      </c>
+      <c r="I28" t="n">
+        <v>95</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="L28" s="35" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>items/chinese-floral-mat-18x24</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>FB draft saved — needs photos added then publish. 3 photos in items/chinese-floral-mat-18x24/.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2416,7 +2472,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
         <is>
@@ -2435,7 +2490,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="34" t="inlineStr">
         <is>

</xml_diff>